<commit_message>
docs(j1): remplace release planning
</commit_message>
<xml_diff>
--- a/docs/perturbations/j1/release-planning.xlsx
+++ b/docs/perturbations/j1/release-planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dadabyun/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E52CAD6-0D70-C244-86D9-F185002AE3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{39EB8486-FA60-C047-8DA9-4BC287B7829B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="780" windowWidth="17120" windowHeight="18920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="600" windowWidth="17120" windowHeight="18920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="161">
   <si>
     <t>A</t>
   </si>
@@ -77,9 +77,6 @@
     <t>n.c.</t>
   </si>
   <si>
-    <t>Produire les 7 artefacts agiles initiaux centrés sur Léa (persona étudiante prioritaire).</t>
-  </si>
-  <si>
     <t>📋 Validation PO 14h00</t>
   </si>
   <si>
@@ -95,15 +92,6 @@
     <t>8-10</t>
   </si>
   <si>
-    <t>Réagir à J1 + sécuriser le socle MVP : F1 compte, F2 upload, impact Mme Lefèvre analysé.</t>
-  </si>
-  <si>
-    <t>US-01, US-02 + analyse US-J1</t>
-  </si>
-  <si>
-    <t>⚡ J1 à 14h · 🟦 Review 18h</t>
-  </si>
-  <si>
     <t>Sprint 2</t>
   </si>
   <si>
@@ -113,9 +101,6 @@
     <t>9h00 – 12h30</t>
   </si>
   <si>
-    <t>Génération quiz F3 avec LLM local Ollama + préparation données de score exploitables ensuite.</t>
-  </si>
-  <si>
     <t>US-03</t>
   </si>
   <si>
@@ -128,15 +113,6 @@
     <t>Mardi PM</t>
   </si>
   <si>
-    <t>10-12</t>
-  </si>
-  <si>
-    <t>Correction, scoring et résultat détaillé : base commune pour Léa et Mme Lefèvre.</t>
-  </si>
-  <si>
-    <t>US-04, US-05, US-J1-01</t>
-  </si>
-  <si>
     <t>🟦 Sprint Review 18h</t>
   </si>
   <si>
@@ -146,12 +122,6 @@
     <t>Mercredi matin</t>
   </si>
   <si>
-    <t>Historique F6 + repérage simple des étudiants en difficulté + sécurité prompt injection J3.</t>
-  </si>
-  <si>
-    <t>US-06, US-J1-02 + patch sécurité</t>
-  </si>
-  <si>
     <t>⚡ Perturbation J3 à 10h</t>
   </si>
   <si>
@@ -161,15 +131,6 @@
     <t>Mercredi PM</t>
   </si>
   <si>
-    <t>Finaliser Release 1 : MVP F1-F6 + slice enseignant minimal + décision RGPD J3-bis.</t>
-  </si>
-  <si>
-    <t>US-12, US-J1-03 + correctifs R1</t>
-  </si>
-  <si>
-    <t>⚡ J3-bis 14h · 🚀 Release 1 17h45</t>
-  </si>
-  <si>
     <t>Sprint 6</t>
   </si>
   <si>
@@ -179,12 +140,6 @@
     <t>8</t>
   </si>
   <si>
-    <t>Release 2 : enrichissements à forte valeur après MVP, dont besoin enseignant J1 priorisé.</t>
-  </si>
-  <si>
-    <t>US-08, US-11, US-J1-04</t>
-  </si>
-  <si>
     <t>⚡ Perturbation J4 à 10h</t>
   </si>
   <si>
@@ -200,12 +155,6 @@
     <t>6-8</t>
   </si>
   <si>
-    <t>Finaliser Release 2 + préparer démo/soutenance + post-mortem J4.</t>
-  </si>
-  <si>
-    <t>US-07, US-10, US-J1-05 + post-mortem</t>
-  </si>
-  <si>
     <t>🚀 Release 2 17h</t>
   </si>
   <si>
@@ -218,19 +167,7 @@
     <t>Selon planning</t>
   </si>
   <si>
-    <t>Pitch + démo live : Léa prioritaire, Mme Lefèvre ajoutée après J1, décisions MoSCoW et compromis expliqués.</t>
-  </si>
-  <si>
-    <t>🎤 Soutenance + Q/R jury</t>
-  </si>
-  <si>
     <t>TOTAL semaine</t>
-  </si>
-  <si>
-    <t>~ 56-64 SP</t>
-  </si>
-  <si>
-    <t>Capacité totale = 203 h-pers. Scope initial ≈56 SP, scope après J1 ≈64 SP : ajout limité, pas de bascule complète vers enseignant.</t>
   </si>
   <si>
     <t>📌 DÉCISION J1</t>
@@ -576,7 +513,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -696,13 +633,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1E1B4B"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FFB45309"/>
       <name val="Calibri"/>
@@ -775,7 +705,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -828,21 +758,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE0E7FF"/>
         <bgColor rgb="FFE0E7FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF2FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2F0D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -947,7 +862,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -966,44 +881,29 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1014,40 +914,13 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1067,31 +940,31 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -1099,10 +972,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
@@ -1761,7 +1634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:I30"/>
+  <dimension ref="B2:I19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1800,361 +1673,83 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="H14" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="I14" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="17">
-        <v>24.5</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I15" s="17" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" ht="70" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="39">
-        <v>28</v>
-      </c>
-      <c r="F16" s="39" t="s">
-        <v>22</v>
-      </c>
-      <c r="G16" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="I16" s="39" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="E17" s="23">
-        <v>24.5</v>
-      </c>
-      <c r="F17" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="H17" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="I17" s="23" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" ht="59" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="E18" s="20">
-        <v>28</v>
-      </c>
-      <c r="F18" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="G18" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="H18" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="I18" s="20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="23">
-        <v>24.5</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="H19" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="I19" s="23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" ht="61" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="40" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="E20" s="41">
-        <v>28</v>
-      </c>
-      <c r="F20" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="G20" s="41" t="s">
-        <v>45</v>
-      </c>
-      <c r="H20" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="I20" s="41" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="42" t="s">
+    <row r="15" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="43" t="s">
+      <c r="C15" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" s="43">
-        <v>24.5</v>
-      </c>
-      <c r="F21" s="43" t="s">
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="50"/>
+    </row>
+    <row r="16" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="G21" s="43" t="s">
+      <c r="C16" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="H21" s="43" t="s">
+      <c r="D16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="50"/>
+      <c r="G16" s="50"/>
+      <c r="H16" s="50"/>
+      <c r="I16" s="50"/>
+    </row>
+    <row r="17" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="I21" s="43" t="s">
+      <c r="C17" s="49" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="22" spans="2:9" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="25" t="s">
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="50"/>
+      <c r="I17" s="50"/>
+    </row>
+    <row r="18" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C18" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="26" t="s">
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
+    </row>
+    <row r="19" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="E22" s="26">
-        <v>21</v>
-      </c>
-      <c r="F22" s="26" t="s">
+      <c r="C19" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="G22" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="H22" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="I22" s="26" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" ht="95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="E23" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="F23" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="H23" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="I23" s="29" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" ht="94" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="44" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="44">
-        <v>203</v>
-      </c>
-      <c r="F24" s="44" t="s">
-        <v>67</v>
-      </c>
-      <c r="G24" s="46" t="s">
-        <v>68</v>
-      </c>
-      <c r="H24" s="45"/>
-      <c r="I24" s="45"/>
-    </row>
-    <row r="26" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="C26" s="63" t="s">
-        <v>70</v>
-      </c>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
-      <c r="I26" s="64"/>
-    </row>
-    <row r="27" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="47" t="s">
-        <v>71</v>
-      </c>
-      <c r="C27" s="63" t="s">
-        <v>72</v>
-      </c>
-      <c r="D27" s="64"/>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="64"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="64"/>
-    </row>
-    <row r="28" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="47" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="63" t="s">
-        <v>74</v>
-      </c>
-      <c r="D28" s="64"/>
-      <c r="E28" s="64"/>
-      <c r="F28" s="64"/>
-      <c r="G28" s="64"/>
-      <c r="H28" s="64"/>
-      <c r="I28" s="64"/>
-    </row>
-    <row r="29" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="47" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="63" t="s">
-        <v>76</v>
-      </c>
-      <c r="D29" s="64"/>
-      <c r="E29" s="64"/>
-      <c r="F29" s="64"/>
-      <c r="G29" s="64"/>
-      <c r="H29" s="64"/>
-      <c r="I29" s="64"/>
-    </row>
-    <row r="30" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="47" t="s">
-        <v>77</v>
-      </c>
-      <c r="C30" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="D30" s="64"/>
-      <c r="E30" s="64"/>
-      <c r="F30" s="64"/>
-      <c r="G30" s="64"/>
-      <c r="H30" s="64"/>
-      <c r="I30" s="64"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="C28:I28"/>
-    <mergeCell ref="C26:I26"/>
-    <mergeCell ref="C29:I29"/>
-    <mergeCell ref="C30:I30"/>
-    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="C17:I17"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="C19:I19"/>
+    <mergeCell ref="C16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2172,17 +1767,17 @@
   <sheetData>
     <row r="2" spans="2:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="7" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="8" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="C5" s="10">
         <v>20</v>
@@ -2190,52 +1785,52 @@
     </row>
     <row r="6" spans="2:3" ht="67" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="9" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="9" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>85</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="9" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="9" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>89</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="9" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="11" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2258,44 +1853,44 @@
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
@@ -2325,292 +1920,292 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="48" t="s">
+      <c r="A10" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="17">
         <v>24.5</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="G10" s="17" t="s">
+      <c r="F10" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="G10" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="35" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="49" t="s">
+      <c r="B11" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="C11" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="D11" s="19">
+        <v>28</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="44" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="21">
+        <v>24.5</v>
+      </c>
+      <c r="E12" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="21">
+      <c r="F12" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="44" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="G11" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="H11" s="20" t="s">
+      <c r="C13" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="19">
+        <v>28</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="21">
+        <v>24.5</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="23">
+        <v>28</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="21">
+        <v>24.5</v>
+      </c>
+      <c r="E16" s="21" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="50" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="24">
-        <v>24.5</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="G12" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="H12" s="23" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="49" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="20" t="s">
+      <c r="F16" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="23">
         <v>21</v>
       </c>
-      <c r="D13" s="21">
-        <v>28</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="F13" s="20" t="s">
-        <v>109</v>
-      </c>
-      <c r="G13" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="H13" s="20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="50" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="24">
-        <v>24.5</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="H14" s="23" t="s">
+      <c r="E17" s="23" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="51" t="s">
+      <c r="F17" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="H17" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="26" t="s">
+    </row>
+    <row r="18" spans="1:8" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="27">
-        <v>28</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="G15" s="26" t="s">
-        <v>181</v>
-      </c>
-      <c r="H15" s="26" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="24">
-        <v>24.5</v>
-      </c>
-      <c r="E16" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="F16" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>180</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="51" t="s">
-        <v>54</v>
-      </c>
-      <c r="B17" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="27">
-        <v>21</v>
-      </c>
-      <c r="E17" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="F17" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="G17" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="H17" s="26" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="52" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="30" t="s">
+      <c r="B18" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="30" t="s">
+      <c r="E18" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="29" t="s">
-        <v>117</v>
-      </c>
-      <c r="G18" s="29" t="s">
-        <v>179</v>
-      </c>
-      <c r="H18" s="29" t="s">
-        <v>118</v>
+      <c r="F18" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="43" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="53" t="s">
-        <v>66</v>
-      </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="53">
+      <c r="A19" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="39">
         <v>203</v>
       </c>
-      <c r="E19" s="53" t="s">
-        <v>119</v>
-      </c>
-      <c r="F19" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
+      <c r="E19" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="33" t="s">
-        <v>71</v>
+      <c r="A22" s="28" t="s">
+        <v>50</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="34" t="s">
-        <v>73</v>
+      <c r="A23" s="29" t="s">
+        <v>52</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="35" t="s">
-        <v>75</v>
+      <c r="A24" s="30" t="s">
+        <v>54</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>124</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="36" t="s">
-        <v>77</v>
+      <c r="A25" s="31" t="s">
+        <v>56</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>125</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2633,505 +2228,505 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="51" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+    </row>
+    <row r="2" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="56" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+    </row>
+    <row r="3" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="41"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="41"/>
+      <c r="L3" s="41"/>
+    </row>
+    <row r="4" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="53" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+    </row>
+    <row r="5" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="53" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+    </row>
+    <row r="6" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="42" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="52"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+    </row>
+    <row r="7" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="41"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41"/>
+      <c r="L7" s="41"/>
+    </row>
+    <row r="8" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+    </row>
+    <row r="9" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="45">
+        <v>0</v>
+      </c>
+      <c r="D9" s="45">
+        <v>0</v>
+      </c>
+      <c r="E9" s="45">
+        <v>56</v>
+      </c>
+      <c r="F9" s="44" t="s">
+        <v>120</v>
+      </c>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+    </row>
+    <row r="10" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="47">
+        <v>8</v>
+      </c>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47">
+        <v>64</v>
+      </c>
+      <c r="F10" s="46" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+    </row>
+    <row r="11" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="45">
+        <v>16</v>
+      </c>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45">
+        <v>64</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+    </row>
+    <row r="12" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="47">
+        <v>22</v>
+      </c>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47">
+        <v>64</v>
+      </c>
+      <c r="F12" s="46" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-    </row>
-    <row r="2" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="67" t="s">
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
+      <c r="K12" s="41"/>
+      <c r="L12" s="41"/>
+    </row>
+    <row r="13" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-    </row>
-    <row r="3" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="55"/>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="55"/>
-    </row>
-    <row r="4" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="56" t="s">
+      <c r="C13" s="45">
+        <v>25</v>
+      </c>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45">
+        <v>64</v>
+      </c>
+      <c r="F13" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="B4" s="65" t="s">
+      <c r="G13" s="41"/>
+      <c r="H13" s="41"/>
+      <c r="I13" s="41"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="41"/>
+    </row>
+    <row r="14" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="46" t="s">
         <v>129</v>
       </c>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-    </row>
-    <row r="5" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="56" t="s">
+      <c r="C14" s="47">
+        <v>30</v>
+      </c>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47">
+        <v>64</v>
+      </c>
+      <c r="F14" s="46" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="65" t="s">
+      <c r="G14" s="41"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41"/>
+      <c r="L14" s="41"/>
+    </row>
+    <row r="15" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="55"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="55"/>
-    </row>
-    <row r="6" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="56" t="s">
+      <c r="C15" s="45">
+        <v>38</v>
+      </c>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45">
+        <v>64</v>
+      </c>
+      <c r="F15" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="B6" s="65" t="s">
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+    </row>
+    <row r="16" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="46" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="55"/>
-      <c r="J6" s="55"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="55"/>
-    </row>
-    <row r="7" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="55"/>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="55"/>
-    </row>
-    <row r="8" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="57" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="57" t="s">
+      <c r="C16" s="47">
+        <v>46</v>
+      </c>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47">
+        <v>64</v>
+      </c>
+      <c r="F16" s="46" t="s">
         <v>134</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="41"/>
+      <c r="L16" s="41"/>
+    </row>
+    <row r="17" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="41"/>
+      <c r="B17" s="41"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="41"/>
+      <c r="L17" s="41"/>
+    </row>
+    <row r="18" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="41"/>
+      <c r="B18" s="41"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="41"/>
+      <c r="L18" s="41"/>
+    </row>
+    <row r="19" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="48" t="s">
         <v>135</v>
       </c>
-      <c r="D8" s="57" t="s">
+      <c r="B19" s="54" t="s">
         <v>136</v>
       </c>
-      <c r="E8" s="57" t="s">
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="55"/>
+      <c r="F19" s="55"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="41"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="41"/>
+      <c r="L19" s="41"/>
+    </row>
+    <row r="20" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="48" t="s">
         <v>137</v>
       </c>
-      <c r="F8" s="57" t="s">
+      <c r="B20" s="54" t="s">
         <v>138</v>
       </c>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="55"/>
-      <c r="J8" s="55"/>
-      <c r="K8" s="55"/>
-      <c r="L8" s="55"/>
-    </row>
-    <row r="9" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="58" t="s">
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="41"/>
+      <c r="L20" s="41"/>
+    </row>
+    <row r="21" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="58" t="s">
+      <c r="B21" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="C9" s="59">
-        <v>0</v>
-      </c>
-      <c r="D9" s="59">
-        <v>0</v>
-      </c>
-      <c r="E9" s="59">
-        <v>56</v>
-      </c>
-      <c r="F9" s="58" t="s">
-        <v>141</v>
-      </c>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="55"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="55"/>
-      <c r="L9" s="55"/>
-    </row>
-    <row r="10" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="60" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="60" t="s">
-        <v>142</v>
-      </c>
-      <c r="C10" s="61">
-        <v>8</v>
-      </c>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61">
-        <v>64</v>
-      </c>
-      <c r="F10" s="60" t="s">
-        <v>143</v>
-      </c>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="55"/>
-      <c r="L10" s="55"/>
-    </row>
-    <row r="11" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="58" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="58" t="s">
-        <v>144</v>
-      </c>
-      <c r="C11" s="59">
-        <v>16</v>
-      </c>
-      <c r="D11" s="59"/>
-      <c r="E11" s="59">
-        <v>64</v>
-      </c>
-      <c r="F11" s="58" t="s">
-        <v>145</v>
-      </c>
-      <c r="G11" s="55"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="55"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="55"/>
-    </row>
-    <row r="12" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="60" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="60" t="s">
-        <v>146</v>
-      </c>
-      <c r="C12" s="61">
-        <v>22</v>
-      </c>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61">
-        <v>64</v>
-      </c>
-      <c r="F12" s="60" t="s">
-        <v>147</v>
-      </c>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="55"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="55"/>
-    </row>
-    <row r="13" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="58" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="58" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" s="59">
-        <v>25</v>
-      </c>
-      <c r="D13" s="59"/>
-      <c r="E13" s="59">
-        <v>64</v>
-      </c>
-      <c r="F13" s="58" t="s">
-        <v>149</v>
-      </c>
-      <c r="G13" s="55"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="55"/>
-      <c r="J13" s="55"/>
-      <c r="K13" s="55"/>
-      <c r="L13" s="55"/>
-    </row>
-    <row r="14" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="60" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" s="60" t="s">
-        <v>150</v>
-      </c>
-      <c r="C14" s="61">
-        <v>30</v>
-      </c>
-      <c r="D14" s="61"/>
-      <c r="E14" s="61">
-        <v>64</v>
-      </c>
-      <c r="F14" s="60" t="s">
-        <v>151</v>
-      </c>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
-      <c r="J14" s="55"/>
-      <c r="K14" s="55"/>
-      <c r="L14" s="55"/>
-    </row>
-    <row r="15" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="58" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="58" t="s">
-        <v>152</v>
-      </c>
-      <c r="C15" s="59">
-        <v>38</v>
-      </c>
-      <c r="D15" s="59"/>
-      <c r="E15" s="59">
-        <v>64</v>
-      </c>
-      <c r="F15" s="58" t="s">
-        <v>153</v>
-      </c>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
-      <c r="J15" s="55"/>
-      <c r="K15" s="55"/>
-      <c r="L15" s="55"/>
-    </row>
-    <row r="16" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="60" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="60" t="s">
-        <v>154</v>
-      </c>
-      <c r="C16" s="61">
-        <v>46</v>
-      </c>
-      <c r="D16" s="61"/>
-      <c r="E16" s="61">
-        <v>64</v>
-      </c>
-      <c r="F16" s="60" t="s">
-        <v>155</v>
-      </c>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
-      <c r="L16" s="55"/>
-    </row>
-    <row r="17" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="55"/>
-      <c r="B17" s="55"/>
-      <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="55"/>
-      <c r="I17" s="55"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="55"/>
-      <c r="L17" s="55"/>
-    </row>
-    <row r="18" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="55"/>
-      <c r="B18" s="55"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="55"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-    </row>
-    <row r="19" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="62" t="s">
-        <v>156</v>
-      </c>
-      <c r="B19" s="68" t="s">
-        <v>157</v>
-      </c>
-      <c r="C19" s="69"/>
-      <c r="D19" s="69"/>
-      <c r="E19" s="69"/>
-      <c r="F19" s="69"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="55"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="55"/>
-      <c r="K19" s="55"/>
-      <c r="L19" s="55"/>
-    </row>
-    <row r="20" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="62" t="s">
-        <v>158</v>
-      </c>
-      <c r="B20" s="68" t="s">
-        <v>159</v>
-      </c>
-      <c r="C20" s="69"/>
-      <c r="D20" s="69"/>
-      <c r="E20" s="69"/>
-      <c r="F20" s="69"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="55"/>
-      <c r="K20" s="55"/>
-      <c r="L20" s="55"/>
-    </row>
-    <row r="21" spans="1:12" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="62" t="s">
-        <v>160</v>
-      </c>
-      <c r="B21" s="68" t="s">
-        <v>161</v>
-      </c>
-      <c r="C21" s="69"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="69"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="55"/>
-      <c r="K21" s="55"/>
-      <c r="L21" s="55"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="41"/>
+      <c r="J21" s="41"/>
+      <c r="K21" s="41"/>
+      <c r="L21" s="41"/>
     </row>
     <row r="22" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="55"/>
-      <c r="B22" s="55"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="55"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="55"/>
-      <c r="G22" s="55"/>
-      <c r="H22" s="55"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="55"/>
-      <c r="K22" s="55"/>
-      <c r="L22" s="55"/>
+      <c r="A22" s="41"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="41"/>
+      <c r="L22" s="41"/>
     </row>
     <row r="23" spans="1:12" ht="24" x14ac:dyDescent="0.3">
-      <c r="A23" s="54"/>
-      <c r="B23" s="54"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54"/>
-      <c r="H23" s="54"/>
+      <c r="A23" s="40"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
     </row>
     <row r="24" spans="1:12" ht="24" x14ac:dyDescent="0.3">
-      <c r="A24" s="54"/>
-      <c r="B24" s="54"/>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="54"/>
-      <c r="G24" s="54"/>
-      <c r="H24" s="54"/>
+      <c r="A24" s="40"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
     </row>
     <row r="25" spans="1:12" ht="24" x14ac:dyDescent="0.3">
-      <c r="A25" s="54"/>
-      <c r="B25" s="54"/>
-      <c r="C25" s="54"/>
-      <c r="D25" s="54"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
+      <c r="A25" s="40"/>
+      <c r="B25" s="40"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
     </row>
     <row r="26" spans="1:12" ht="24" x14ac:dyDescent="0.3">
-      <c r="A26" s="54"/>
-      <c r="B26" s="54"/>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="E26" s="54"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54"/>
+      <c r="A26" s="40"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="40"/>
     </row>
     <row r="27" spans="1:12" ht="24" x14ac:dyDescent="0.3">
-      <c r="A27" s="54"/>
-      <c r="B27" s="54"/>
-      <c r="C27" s="54"/>
-      <c r="D27" s="54"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="54"/>
-      <c r="G27" s="54"/>
-      <c r="H27" s="54"/>
+      <c r="A27" s="40"/>
+      <c r="B27" s="40"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
     </row>
     <row r="28" spans="1:12" ht="24" x14ac:dyDescent="0.3">
-      <c r="A28" s="54"/>
-      <c r="B28" s="54"/>
-      <c r="C28" s="54"/>
-      <c r="D28" s="54"/>
-      <c r="E28" s="54"/>
-      <c r="F28" s="54"/>
-      <c r="G28" s="54"/>
-      <c r="H28" s="54"/>
+      <c r="A28" s="40"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B20:F20"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -3151,106 +2746,106 @@
   <sheetData>
     <row r="2" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B3" s="8" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="15"/>
       <c r="B5" s="15" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>165</v>
+        <v>144</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>168</v>
-      </c>
-      <c r="D6" s="37"/>
+      <c r="B6" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="32"/>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>169</v>
-      </c>
-      <c r="D7" s="37"/>
+      <c r="B7" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="D7" s="32"/>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>170</v>
-      </c>
-      <c r="D8" s="37"/>
+      <c r="B8" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="32"/>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>171</v>
-      </c>
-      <c r="D9" s="37"/>
+      <c r="B9" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>150</v>
+      </c>
+      <c r="D9" s="32"/>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="D10" s="37"/>
+      <c r="B10" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>151</v>
+      </c>
+      <c r="D10" s="32"/>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C11" s="37" t="s">
-        <v>173</v>
-      </c>
-      <c r="D11" s="37"/>
+      <c r="B11" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" s="32"/>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>174</v>
-      </c>
-      <c r="D12" s="37"/>
+      <c r="B12" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>153</v>
+      </c>
+      <c r="D12" s="32"/>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C13" s="37" t="s">
-        <v>175</v>
-      </c>
-      <c r="D13" s="37"/>
+      <c r="B13" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="D13" s="32"/>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="37" t="s">
-        <v>176</v>
-      </c>
-      <c r="C14" s="37" t="s">
-        <v>177</v>
-      </c>
-      <c r="D14" s="37"/>
+      <c r="B14" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>156</v>
+      </c>
+      <c r="D14" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>